<commit_message>
Add screenshots of bugs and Jira bug reports
</commit_message>
<xml_diff>
--- a/manual_testing/SauceDemo_bug_report.xlsx
+++ b/manual_testing/SauceDemo_bug_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandra\Documents\IT Bootcamp\Projekat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0544DF-5F0C-410F-8815-0FCD1CA659C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DDAC5D-3C21-4F70-9CE4-F157FAEAE479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="1080" windowWidth="26295" windowHeight="15420" activeTab="3" xr2:uid="{126E7B82-619F-444B-888F-0D58DA0BEF2A}"/>
+    <workbookView xWindow="7725" yWindow="2355" windowWidth="12960" windowHeight="15420" activeTab="3" xr2:uid="{126E7B82-619F-444B-888F-0D58DA0BEF2A}"/>
   </bookViews>
   <sheets>
     <sheet name="SD-BR-1" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="71">
   <si>
     <t>Step no.</t>
   </si>
@@ -218,15 +218,9 @@
     <t>Critical</t>
   </si>
   <si>
-    <t>It is possible to click "Continue" button on Cart page with empty cart proceeding to Checkout-step-one page where is posible to click on "Continue" button that leads to Checkout-step-two page and click "Finish" button to succesfully finish purchase with zero items and total amount of $0.00. Cart-emptiness validation is missing at multiple checkpoints in the checkout flow, not just on the initial Cart page.</t>
-  </si>
-  <si>
     <t>It is possible to complete the purchase with numbers in First name text field</t>
   </si>
   <si>
-    <t>User is logged in as “standard_user” and is on Checkout-step-one page</t>
-  </si>
-  <si>
     <t>It is possible to complete the purchase with numbers in Last name text field</t>
   </si>
   <si>
@@ -248,12 +242,6 @@
     <t>Input numbers in Last name text field (input:  4321 )</t>
   </si>
   <si>
-    <t xml:space="preserve">Finish button cannot be clicked and user cannot continue to paying, , proper Error message is displayed </t>
-  </si>
-  <si>
-    <t>Continue button can be clicked and user is on Checkout-complete page, Success message is shown</t>
-  </si>
-  <si>
     <t>OS</t>
   </si>
   <si>
@@ -270,6 +258,24 @@
   </si>
   <si>
     <t>It is possible to complete purchase with numbers in Last name text field, indicating that input validation is not properly inplemented. Connected to SD_BR_3 (possible to put numbers in First name field), and the third field (zipcode) was also observed and it does not validate input indicating that problem is wider and across the entire information form which could result in failed order delivery.</t>
+  </si>
+  <si>
+    <t>It is possible to click "Checkout" button on Cart page with empty cart proceeding to Checkout-step-one page where is posible to click on "Continue" button that leads to Checkout-step-two page and click "Finish" button to succesfully finish purchase with zero items and total amount of $0.00. Cart-emptiness validation is missing at multiple checkpoints in the checkout flow, not just on the initial Cart page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continue button cannot be clicked and user cannot continue to paying, proper Error message is displayed </t>
+  </si>
+  <si>
+    <t>Continue</t>
+  </si>
+  <si>
+    <t>Click on the  Continue button</t>
+  </si>
+  <si>
+    <t>User is logged in as “standard_user” and is on Cart page containing one item</t>
+  </si>
+  <si>
+    <t>Continue button can be clicked and user is on Checkout-step-two page</t>
   </si>
 </sst>
 </file>
@@ -1772,25 +1778,25 @@
     </row>
     <row r="31" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="60" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D31" s="34"/>
     </row>
     <row r="32" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D32" s="34"/>
     </row>
     <row r="33" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="61" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D33" s="34"/>
     </row>
     <row r="34" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D34" s="34"/>
     </row>
@@ -1799,17 +1805,17 @@
       <c r="D35" s="35"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C31">
+    <cfRule type="duplicateValues" dxfId="15" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23 C25:D25">
-    <cfRule type="duplicateValues" dxfId="15" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="duplicateValues" dxfId="14" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 H3:H4">
-    <cfRule type="duplicateValues" dxfId="13" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1919,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="51" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D7" s="43"/>
       <c r="E7" s="16" t="s">
@@ -2108,7 +2114,7 @@
     </row>
     <row r="28" spans="2:6" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="49" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="D28" s="32"/>
       <c r="E28" s="2"/>
@@ -2123,25 +2129,25 @@
     </row>
     <row r="31" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="60" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D31" s="34"/>
     </row>
     <row r="32" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D32" s="34"/>
     </row>
     <row r="33" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="61" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D33" s="34"/>
     </row>
     <row r="34" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D34" s="34"/>
     </row>
@@ -2150,17 +2156,17 @@
       <c r="D35" s="35"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C31">
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23 C25:D25">
-    <cfRule type="duplicateValues" dxfId="12" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="duplicateValues" dxfId="11" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 H3:H4">
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2207,7 +2213,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D3" s="37"/>
       <c r="E3" s="29" t="s">
@@ -2239,7 +2245,7 @@
     <row r="5" spans="2:8" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="24"/>
       <c r="C5" s="14" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D5" s="38"/>
       <c r="E5" s="29"/>
@@ -2271,8 +2277,8 @@
       <c r="B7" s="7">
         <v>1</v>
       </c>
-      <c r="C7" s="33" t="s">
-        <v>55</v>
+      <c r="C7" s="59" t="s">
+        <v>54</v>
       </c>
       <c r="D7" s="43"/>
       <c r="E7" s="16" t="s">
@@ -2285,8 +2291,8 @@
       <c r="B8" s="8">
         <v>2</v>
       </c>
-      <c r="C8" s="59" t="s">
-        <v>56</v>
+      <c r="C8" s="52" t="s">
+        <v>55</v>
       </c>
       <c r="D8" s="44"/>
       <c r="E8" s="6" t="s">
@@ -2303,8 +2309,8 @@
       <c r="B9" s="8">
         <v>3</v>
       </c>
-      <c r="C9" s="52" t="s">
-        <v>57</v>
+      <c r="C9" s="33" t="s">
+        <v>56</v>
       </c>
       <c r="D9" s="45"/>
       <c r="E9" s="16" t="s">
@@ -2321,10 +2327,12 @@
       <c r="B10" s="8">
         <v>4</v>
       </c>
-      <c r="C10" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="45"/>
+      <c r="C10" s="62" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>67</v>
+      </c>
       <c r="E10" s="6" t="s">
         <v>8</v>
       </c>
@@ -2333,8 +2341,8 @@
       <c r="B11" s="8">
         <v>5</v>
       </c>
-      <c r="C11" s="51" t="s">
-        <v>43</v>
+      <c r="C11" s="62" t="s">
+        <v>47</v>
       </c>
       <c r="D11" s="46"/>
       <c r="E11" s="14" t="s">
@@ -2345,9 +2353,7 @@
       <c r="B12" s="8">
         <v>6</v>
       </c>
-      <c r="C12" s="62" t="s">
-        <v>47</v>
-      </c>
+      <c r="C12" s="62"/>
       <c r="D12" s="63"/>
       <c r="E12" s="5"/>
     </row>
@@ -2437,7 +2443,7 @@
     </row>
     <row r="24" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="54" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D24" s="32"/>
     </row>
@@ -2449,7 +2455,7 @@
     </row>
     <row r="26" spans="2:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="54" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D26" s="32"/>
     </row>
@@ -2461,7 +2467,7 @@
     </row>
     <row r="28" spans="2:6" ht="107.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="49" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D28" s="32"/>
       <c r="E28" s="2"/>
@@ -2476,25 +2482,25 @@
     </row>
     <row r="31" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="60" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D31" s="34"/>
     </row>
     <row r="32" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D32" s="34"/>
     </row>
     <row r="33" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="61" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D33" s="34"/>
     </row>
     <row r="34" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D34" s="34"/>
     </row>
@@ -2503,17 +2509,17 @@
       <c r="D35" s="35"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C31">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23 C25:D25">
-    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 H3:H4">
-    <cfRule type="duplicateValues" dxfId="7" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2560,7 +2566,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D3" s="37"/>
       <c r="E3" s="29" t="s">
@@ -2592,7 +2598,7 @@
     <row r="5" spans="2:8" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="24"/>
       <c r="C5" s="14" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D5" s="38"/>
       <c r="E5" s="29"/>
@@ -2625,7 +2631,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D7" s="43"/>
       <c r="E7" s="16" t="s">
@@ -2639,7 +2645,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D8" s="44"/>
       <c r="E8" s="6" t="s">
@@ -2657,7 +2663,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="51" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D9" s="45"/>
       <c r="E9" s="16" t="s">
@@ -2675,7 +2681,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D10" s="45"/>
       <c r="E10" s="6" t="s">
@@ -2790,7 +2796,7 @@
     </row>
     <row r="24" spans="2:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="54" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D24" s="32"/>
     </row>
@@ -2802,7 +2808,7 @@
     </row>
     <row r="26" spans="2:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="54" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D26" s="32"/>
     </row>
@@ -2814,7 +2820,7 @@
     </row>
     <row r="28" spans="2:6" ht="106.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="49" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D28" s="32"/>
       <c r="E28" s="2"/>
@@ -2829,25 +2835,25 @@
     </row>
     <row r="31" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="60" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D31" s="34"/>
     </row>
     <row r="32" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="20" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D32" s="34"/>
     </row>
     <row r="33" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="61" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D33" s="34"/>
     </row>
     <row r="34" spans="3:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D34" s="34"/>
     </row>
@@ -2856,17 +2862,17 @@
       <c r="D35" s="35"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C31">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23 C25:D25">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 H3:H4">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>